<commit_message>
translation of the paper
</commit_message>
<xml_diff>
--- a/Data/data_four_species.xlsx
+++ b/Data/data_four_species.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e91640961c0a8f3d/Рабочий стол/Python_repos/Python_projects_ICG_SB_RAS/Four_host_species_OF/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Yaroslav\Desktop\Python_repos\Python_projects_ICG_SB_RAS\Four_host_species_OF\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="277" documentId="13_ncr:1_{515605E3-398A-4E11-A388-A32BC0C2CB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5264230-0E92-4167-A53F-A8C2BD870548}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E5330AC-0222-403C-B8D2-A5AA3BBAECDA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15360" yWindow="0" windowWidth="15360" windowHeight="16680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="fluke_data" sheetId="1" r:id="rId1"/>
@@ -160,7 +160,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -285,11 +285,29 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -308,10 +326,13 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -592,7 +613,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
@@ -976,7 +997,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>1</v>
       </c>
@@ -999,7 +1020,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>2</v>
       </c>
@@ -1022,7 +1043,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>3</v>
       </c>
@@ -1045,7 +1066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>4</v>
       </c>
@@ -1068,7 +1089,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>5</v>
       </c>
@@ -1091,464 +1112,493 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="1">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22" s="20">
         <v>1</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D22" s="1">
-        <v>0</v>
-      </c>
-      <c r="E22" s="1">
-        <v>0</v>
-      </c>
-      <c r="F22" s="1">
-        <v>0</v>
-      </c>
-      <c r="G22" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="1">
+      <c r="B22" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D22" s="20">
+        <v>0</v>
+      </c>
+      <c r="E22" s="20">
+        <v>0</v>
+      </c>
+      <c r="F22" s="20">
+        <v>0</v>
+      </c>
+      <c r="G22" s="20">
+        <v>0</v>
+      </c>
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23" s="20">
         <v>2</v>
       </c>
-      <c r="B23" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D23" s="1">
-        <v>0</v>
-      </c>
-      <c r="E23" s="1">
-        <v>0</v>
-      </c>
-      <c r="F23" s="1">
-        <v>0</v>
-      </c>
-      <c r="G23" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="1">
-        <v>3</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D24" s="1">
-        <v>0</v>
-      </c>
-      <c r="E24" s="1">
-        <v>0</v>
-      </c>
-      <c r="F24" s="1">
-        <v>0</v>
-      </c>
-      <c r="G24" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="1">
-        <v>4</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D25" s="1">
-        <v>0</v>
-      </c>
-      <c r="E25" s="1">
-        <v>0</v>
-      </c>
-      <c r="F25" s="1">
-        <v>0</v>
-      </c>
-      <c r="G25" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="1">
-        <v>5</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C26" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D26" s="1">
-        <v>0</v>
-      </c>
-      <c r="E26" s="1">
-        <v>0</v>
-      </c>
-      <c r="F26" s="1">
-        <v>0</v>
-      </c>
-      <c r="G26" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="1">
+      <c r="B23" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" s="20">
+        <v>0</v>
+      </c>
+      <c r="E23" s="20">
+        <v>0</v>
+      </c>
+      <c r="F23" s="20">
+        <v>0</v>
+      </c>
+      <c r="G23" s="20">
+        <v>0</v>
+      </c>
+      <c r="H23" s="20"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24" s="20">
+        <v>3</v>
+      </c>
+      <c r="B24" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D24" s="20">
+        <v>0</v>
+      </c>
+      <c r="E24" s="20">
+        <v>0</v>
+      </c>
+      <c r="F24" s="20">
+        <v>0</v>
+      </c>
+      <c r="G24" s="20">
+        <v>0</v>
+      </c>
+      <c r="H24" s="20"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25" s="20">
+        <v>4</v>
+      </c>
+      <c r="B25" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D25" s="20">
+        <v>0</v>
+      </c>
+      <c r="E25" s="20">
+        <v>0</v>
+      </c>
+      <c r="F25" s="20">
+        <v>0</v>
+      </c>
+      <c r="G25" s="20">
+        <v>0</v>
+      </c>
+      <c r="H25" s="20"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26" s="21">
+        <v>5</v>
+      </c>
+      <c r="B26" s="21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D26" s="21">
+        <v>0</v>
+      </c>
+      <c r="E26" s="21">
+        <v>0</v>
+      </c>
+      <c r="F26" s="21">
+        <v>0</v>
+      </c>
+      <c r="G26" s="21">
+        <v>0</v>
+      </c>
+      <c r="H26" s="21"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" s="20">
         <v>1</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C27" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D27" s="1">
-        <v>0</v>
-      </c>
-      <c r="E27" s="1">
+      <c r="C27" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D27" s="20">
+        <v>0</v>
+      </c>
+      <c r="E27" s="20">
         <v>0.2</v>
       </c>
-      <c r="F27" s="1">
-        <v>0</v>
-      </c>
-      <c r="G27" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="1">
+      <c r="F27" s="20">
+        <v>0</v>
+      </c>
+      <c r="G27" s="20">
+        <v>0</v>
+      </c>
+      <c r="H27" s="20"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28" s="20">
         <v>2</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D28" s="1">
+      <c r="C28" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D28" s="20">
         <v>1</v>
       </c>
-      <c r="E28" s="1">
+      <c r="E28" s="20">
         <v>0.7</v>
       </c>
-      <c r="F28" s="1">
+      <c r="F28" s="20">
         <v>35</v>
       </c>
-      <c r="G28" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="1">
-        <v>3</v>
-      </c>
-      <c r="B29" s="1" t="s">
+      <c r="G28" s="20">
+        <v>0</v>
+      </c>
+      <c r="H28" s="20"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29" s="20">
+        <v>3</v>
+      </c>
+      <c r="B29" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C29" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D29" s="1">
+      <c r="C29" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D29" s="20">
         <v>1</v>
       </c>
-      <c r="E29" s="1">
+      <c r="E29" s="20">
         <v>0.9</v>
       </c>
-      <c r="F29" s="1">
+      <c r="F29" s="20">
         <v>60</v>
       </c>
-      <c r="G29" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="1">
-        <v>4</v>
-      </c>
-      <c r="B30" s="1" t="s">
+      <c r="G29" s="20">
+        <v>0</v>
+      </c>
+      <c r="H29" s="20"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A30" s="20">
+        <v>4</v>
+      </c>
+      <c r="B30" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="C30" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D30" s="1">
+      <c r="C30" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D30" s="20">
         <v>2</v>
       </c>
-      <c r="E30" s="1">
+      <c r="E30" s="20">
         <v>1.4</v>
       </c>
-      <c r="F30" s="1">
-        <v>0</v>
-      </c>
-      <c r="G30" s="1">
+      <c r="F30" s="20">
+        <v>0</v>
+      </c>
+      <c r="G30" s="20">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="1">
-        <v>5</v>
-      </c>
-      <c r="B31" s="1" t="s">
+      <c r="H30" s="20"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A31" s="21">
+        <v>5</v>
+      </c>
+      <c r="B31" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D31" s="1">
-        <v>3</v>
-      </c>
-      <c r="E31" s="1">
+      <c r="C31" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="21">
+        <v>3</v>
+      </c>
+      <c r="E31" s="21">
         <v>1.9</v>
       </c>
-      <c r="F31" s="1">
+      <c r="F31" s="21">
         <v>19</v>
       </c>
-      <c r="G31" s="1">
+      <c r="G31" s="21">
         <v>2.2000000000000002</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="1">
+      <c r="H31" s="21">
+        <f>AVERAGE(G27:G31)</f>
+        <v>0.48000000000000009</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A32" s="22">
         <v>1</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="22" t="s">
         <v>7</v>
       </c>
-      <c r="C32" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D32" s="1">
-        <v>3</v>
-      </c>
-      <c r="E32" s="1">
+      <c r="C32" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D32" s="22">
+        <v>3</v>
+      </c>
+      <c r="E32" s="22">
         <v>0.8</v>
       </c>
-      <c r="F32" s="1">
-        <v>0</v>
-      </c>
-      <c r="G32" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="1">
+      <c r="F32" s="22">
+        <v>0</v>
+      </c>
+      <c r="G32" s="22">
+        <v>0</v>
+      </c>
+      <c r="H32" s="22"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="20">
         <v>2</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D33" s="1">
-        <v>5</v>
-      </c>
-      <c r="E33" s="1">
+      <c r="C33" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="20">
+        <v>5</v>
+      </c>
+      <c r="E33" s="20">
         <v>0.9</v>
       </c>
-      <c r="F33" s="1">
+      <c r="F33" s="20">
         <v>180</v>
       </c>
-      <c r="G33" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="1">
-        <v>3</v>
-      </c>
-      <c r="B34" s="1" t="s">
+      <c r="G33" s="20">
+        <v>0</v>
+      </c>
+      <c r="H33" s="20"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="20">
+        <v>3</v>
+      </c>
+      <c r="B34" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C34" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D34" s="1">
+      <c r="C34" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="20">
         <v>7</v>
       </c>
-      <c r="E34" s="1">
+      <c r="E34" s="20">
         <v>3.9</v>
       </c>
-      <c r="F34" s="1">
+      <c r="F34" s="20">
         <v>220</v>
       </c>
-      <c r="G34" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="1">
-        <v>4</v>
-      </c>
-      <c r="B35" s="1" t="s">
+      <c r="G34" s="20">
+        <v>0</v>
+      </c>
+      <c r="H34" s="20"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="20">
+        <v>4</v>
+      </c>
+      <c r="B35" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C35" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D35" s="1">
+      <c r="C35" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D35" s="20">
         <v>9</v>
       </c>
-      <c r="E35" s="1">
+      <c r="E35" s="20">
         <v>6</v>
       </c>
-      <c r="F35" s="1">
+      <c r="F35" s="20">
         <v>80</v>
       </c>
-      <c r="G35" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="1">
-        <v>5</v>
-      </c>
-      <c r="B36" s="1" t="s">
+      <c r="G35" s="20">
+        <v>4</v>
+      </c>
+      <c r="H35" s="20"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="21">
+        <v>5</v>
+      </c>
+      <c r="B36" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D36" s="1">
+      <c r="C36" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" s="21">
         <v>14</v>
       </c>
-      <c r="E36" s="1">
+      <c r="E36" s="21">
         <v>7</v>
       </c>
-      <c r="F36" s="1">
+      <c r="F36" s="21">
         <v>99</v>
       </c>
-      <c r="G36" s="1">
+      <c r="G36" s="21">
         <v>23</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="1">
+      <c r="H36" s="21">
+        <f>AVERAGE(G32:G36)</f>
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="22">
         <v>1</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="C37" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D37" s="1">
+      <c r="C37" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D37" s="22">
         <v>32</v>
       </c>
-      <c r="E37" s="1">
+      <c r="E37" s="22">
         <v>3.8</v>
       </c>
-      <c r="F37" s="1">
+      <c r="F37" s="22">
         <v>1050</v>
       </c>
-      <c r="G37" s="1">
+      <c r="G37" s="22">
         <v>25</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="1">
+      <c r="H37" s="22"/>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="20">
         <v>2</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C38" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D38" s="1">
+      <c r="C38" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D38" s="20">
         <v>35</v>
       </c>
-      <c r="E38" s="1">
+      <c r="E38" s="20">
         <v>4.5</v>
       </c>
-      <c r="F38" s="1">
+      <c r="F38" s="20">
         <v>1200</v>
       </c>
-      <c r="G38" s="1">
+      <c r="G38" s="20">
         <v>30</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" s="1">
-        <v>3</v>
-      </c>
-      <c r="B39" s="1" t="s">
+      <c r="H38" s="20"/>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="20">
+        <v>3</v>
+      </c>
+      <c r="B39" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C39" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D39" s="1">
+      <c r="C39" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D39" s="20">
         <v>36</v>
       </c>
-      <c r="E39" s="1">
+      <c r="E39" s="20">
         <v>4.7</v>
       </c>
-      <c r="F39" s="1">
+      <c r="F39" s="20">
         <v>1250</v>
       </c>
-      <c r="G39" s="1">
+      <c r="G39" s="20">
         <v>33</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" s="1">
-        <v>4</v>
-      </c>
-      <c r="B40" s="1" t="s">
+      <c r="H39" s="20"/>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="20">
+        <v>4</v>
+      </c>
+      <c r="B40" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C40" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D40" s="1">
+      <c r="C40" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" s="20">
         <v>44</v>
       </c>
-      <c r="E40" s="1">
+      <c r="E40" s="20">
         <v>5.2</v>
       </c>
-      <c r="F40" s="1">
+      <c r="F40" s="20">
         <v>1400</v>
       </c>
-      <c r="G40" s="1">
+      <c r="G40" s="20">
         <v>39</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="1">
-        <v>5</v>
-      </c>
-      <c r="B41" s="1" t="s">
+      <c r="H40" s="20"/>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="21">
+        <v>5</v>
+      </c>
+      <c r="B41" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D41" s="1">
+      <c r="C41" s="21" t="s">
+        <v>5</v>
+      </c>
+      <c r="D41" s="21">
         <v>49</v>
       </c>
-      <c r="E41" s="1">
+      <c r="E41" s="21">
         <v>5.6</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F41" s="21">
         <v>1650</v>
       </c>
-      <c r="G41" s="1">
+      <c r="G41" s="21">
         <v>49</v>
+      </c>
+      <c r="H41" s="21">
+        <f>AVERAGE(G37:G41)</f>
+        <v>35.200000000000003</v>
       </c>
     </row>
   </sheetData>
@@ -1565,7 +1615,7 @@
     <col min="1" max="1" width="8.88671875" style="17"/>
     <col min="2" max="2" width="13.6640625" style="17" customWidth="1"/>
     <col min="3" max="3" width="16.109375" style="17" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" style="19" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" style="18" customWidth="1"/>
     <col min="5" max="5" width="16.21875" style="17" customWidth="1"/>
     <col min="6" max="6" width="10.21875" style="17" customWidth="1"/>
     <col min="7" max="8" width="12" style="17" customWidth="1"/>
@@ -1590,7 +1640,7 @@
       <c r="C1" s="17" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="18" t="s">
         <v>13</v>
       </c>
       <c r="E1" s="17" t="s">
@@ -1616,7 +1666,7 @@
       <c r="C2" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="19">
+      <c r="D2" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E2" s="17">
@@ -1642,7 +1692,7 @@
       <c r="C3" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="19">
+      <c r="D3" s="18">
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="E3" s="17">
@@ -1668,7 +1718,7 @@
       <c r="C4" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="18">
         <v>3.0000000000000001E-5</v>
       </c>
       <c r="E4" s="17">
@@ -1694,7 +1744,7 @@
       <c r="C5" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="18">
         <v>4.0000000000000003E-5</v>
       </c>
       <c r="E5" s="17">
@@ -1720,7 +1770,7 @@
       <c r="C6" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="18">
         <v>5.0000000000000002E-5</v>
       </c>
       <c r="E6" s="17">
@@ -1746,7 +1796,7 @@
       <c r="C7" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="18">
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="E7" s="17">
@@ -1772,7 +1822,7 @@
       <c r="C8" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E8" s="17">
@@ -1798,7 +1848,7 @@
       <c r="C9" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="18">
         <v>8.0000000000000007E-5</v>
       </c>
       <c r="E9" s="17">
@@ -1824,7 +1874,7 @@
       <c r="C10" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="18">
         <v>1.2E-5</v>
       </c>
       <c r="E10" s="17">
@@ -1850,7 +1900,7 @@
       <c r="C11" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="18">
         <v>3.1000000000000001E-5</v>
       </c>
       <c r="E11" s="17">
@@ -1876,7 +1926,7 @@
       <c r="C12" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="18">
         <v>6.9999999999999994E-5</v>
       </c>
       <c r="E12" s="17">
@@ -1902,7 +1952,7 @@
       <c r="C13" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D13" s="19">
+      <c r="D13" s="18">
         <v>9.0000000000000006E-5</v>
       </c>
       <c r="E13" s="17">
@@ -1928,7 +1978,7 @@
       <c r="C14" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D14" s="19">
+      <c r="D14" s="18">
         <v>1.5E-5</v>
       </c>
       <c r="E14" s="17">
@@ -1954,7 +2004,7 @@
       <c r="C15" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D15" s="19">
+      <c r="D15" s="18">
         <v>1.112E-5</v>
       </c>
       <c r="E15" s="17">
@@ -1980,7 +2030,7 @@
       <c r="C16" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="19">
+      <c r="D16" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E16" s="17">
@@ -2006,7 +2056,7 @@
       <c r="C17" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D17" s="19">
+      <c r="D17" s="18">
         <v>5.0000000000000002E-5</v>
       </c>
       <c r="E17" s="17">
@@ -2032,7 +2082,7 @@
       <c r="C18" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D18" s="19">
+      <c r="D18" s="18">
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="E18" s="17">
@@ -2058,7 +2108,7 @@
       <c r="C19" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D19" s="19">
+      <c r="D19" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E19" s="17">
@@ -2084,7 +2134,7 @@
       <c r="C20" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="18">
         <v>8.0000000000000007E-5</v>
       </c>
       <c r="E20" s="17">
@@ -2110,7 +2160,7 @@
       <c r="C21" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D21" s="19">
+      <c r="D21" s="18">
         <v>1.2E-5</v>
       </c>
       <c r="E21" s="17">
@@ -2136,7 +2186,7 @@
       <c r="C22" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D22" s="19">
+      <c r="D22" s="18">
         <v>3</v>
       </c>
       <c r="E22" s="17">
@@ -2162,7 +2212,7 @@
       <c r="C23" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D23" s="19">
+      <c r="D23" s="18">
         <v>3.2</v>
       </c>
       <c r="E23" s="17">
@@ -2188,7 +2238,7 @@
       <c r="C24" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D24" s="19">
+      <c r="D24" s="18">
         <v>4.0999999999999996</v>
       </c>
       <c r="E24" s="17">
@@ -2214,7 +2264,7 @@
       <c r="C25" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D25" s="19">
+      <c r="D25" s="18">
         <v>4.5</v>
       </c>
       <c r="E25" s="17">
@@ -2240,7 +2290,7 @@
       <c r="C26" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D26" s="19">
+      <c r="D26" s="18">
         <v>9.3000000000000007</v>
       </c>
       <c r="E26" s="17">
@@ -2266,7 +2316,7 @@
       <c r="C27" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D27" s="19">
+      <c r="D27" s="18">
         <v>3.4</v>
       </c>
       <c r="E27" s="17">
@@ -2292,7 +2342,7 @@
       <c r="C28" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D28" s="19">
+      <c r="D28" s="18">
         <v>5.2</v>
       </c>
       <c r="E28" s="17">
@@ -2318,7 +2368,7 @@
       <c r="C29" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D29" s="19">
+      <c r="D29" s="18">
         <v>5.6</v>
       </c>
       <c r="E29" s="17">
@@ -2344,7 +2394,7 @@
       <c r="C30" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D30" s="19">
+      <c r="D30" s="18">
         <v>5.9</v>
       </c>
       <c r="E30" s="17">
@@ -2370,7 +2420,7 @@
       <c r="C31" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D31" s="19">
+      <c r="D31" s="18">
         <v>9.4</v>
       </c>
       <c r="E31" s="17">
@@ -2396,7 +2446,7 @@
       <c r="C32" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D32" s="19">
+      <c r="D32" s="18">
         <v>6.9999999999999994E-5</v>
       </c>
       <c r="E32" s="17">
@@ -2422,7 +2472,7 @@
       <c r="C33" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D33" s="19">
+      <c r="D33" s="18">
         <v>9.0000000000000006E-5</v>
       </c>
       <c r="E33" s="17">
@@ -2448,7 +2498,7 @@
       <c r="C34" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D34" s="19">
+      <c r="D34" s="18">
         <v>1.5E-5</v>
       </c>
       <c r="E34" s="17">
@@ -2474,7 +2524,7 @@
       <c r="C35" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D35" s="19">
+      <c r="D35" s="18">
         <v>1.112E-5</v>
       </c>
       <c r="E35" s="17">
@@ -2500,7 +2550,7 @@
       <c r="C36" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D36" s="19">
+      <c r="D36" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E36" s="17">
@@ -2526,7 +2576,7 @@
       <c r="C37" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D37" s="19">
+      <c r="D37" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E37" s="17">
@@ -2552,7 +2602,7 @@
       <c r="C38" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D38" s="19">
+      <c r="D38" s="18">
         <v>1.8</v>
       </c>
       <c r="E38" s="17">
@@ -2578,7 +2628,7 @@
       <c r="C39" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D39" s="19">
+      <c r="D39" s="18">
         <v>5.7</v>
       </c>
       <c r="E39" s="17">
@@ -2604,7 +2654,7 @@
       <c r="C40" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D40" s="19">
+      <c r="D40" s="18">
         <v>6.9</v>
       </c>
       <c r="E40" s="17">
@@ -2630,7 +2680,7 @@
       <c r="C41" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D41" s="19">
+      <c r="D41" s="18">
         <v>7</v>
       </c>
       <c r="E41" s="17">
@@ -2656,7 +2706,7 @@
       <c r="C42" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D42" s="19">
+      <c r="D42" s="18">
         <v>1.3</v>
       </c>
       <c r="E42" s="17">
@@ -2682,7 +2732,7 @@
       <c r="C43" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D43" s="19">
+      <c r="D43" s="18">
         <v>2.6</v>
       </c>
       <c r="E43" s="17">
@@ -2708,7 +2758,7 @@
       <c r="C44" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D44" s="19">
+      <c r="D44" s="18">
         <v>3.1</v>
       </c>
       <c r="E44" s="17">
@@ -2734,7 +2784,7 @@
       <c r="C45" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D45" s="19">
+      <c r="D45" s="18">
         <v>6</v>
       </c>
       <c r="E45" s="17">
@@ -2760,7 +2810,7 @@
       <c r="C46" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D46" s="19">
+      <c r="D46" s="18">
         <v>12.7</v>
       </c>
       <c r="E46" s="17">
@@ -2786,7 +2836,7 @@
       <c r="C47" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D47" s="19">
+      <c r="D47" s="18">
         <v>1.0000000000000001E-5</v>
       </c>
       <c r="E47" s="17">
@@ -2812,7 +2862,7 @@
       <c r="C48" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D48" s="19">
+      <c r="D48" s="18">
         <v>2.0000000000000002E-5</v>
       </c>
       <c r="E48" s="17">
@@ -2838,7 +2888,7 @@
       <c r="C49" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D49" s="19">
+      <c r="D49" s="18">
         <v>3.0000000000000001E-5</v>
       </c>
       <c r="E49" s="17">
@@ -2864,7 +2914,7 @@
       <c r="C50" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D50" s="19">
+      <c r="D50" s="18">
         <v>4.0000000000000003E-5</v>
       </c>
       <c r="E50" s="17">
@@ -2890,7 +2940,7 @@
       <c r="C51" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="D51" s="19">
+      <c r="D51" s="18">
         <v>5.0000000000000002E-5</v>
       </c>
       <c r="E51" s="17">
@@ -2916,7 +2966,7 @@
       <c r="C52" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D52" s="19">
+      <c r="D52" s="18">
         <v>6.2</v>
       </c>
       <c r="E52" s="17">
@@ -2942,7 +2992,7 @@
       <c r="C53" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D53" s="19">
+      <c r="D53" s="18">
         <v>6.5</v>
       </c>
       <c r="E53" s="17">
@@ -2968,7 +3018,7 @@
       <c r="C54" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D54" s="19">
+      <c r="D54" s="18">
         <v>6.8</v>
       </c>
       <c r="E54" s="17">
@@ -2994,7 +3044,7 @@
       <c r="C55" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D55" s="19">
+      <c r="D55" s="18">
         <v>7.4</v>
       </c>
       <c r="E55" s="17">
@@ -3020,7 +3070,7 @@
       <c r="C56" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="D56" s="19">
+      <c r="D56" s="18">
         <v>8</v>
       </c>
       <c r="E56" s="17">
@@ -3046,7 +3096,7 @@
       <c r="C57" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D57" s="19">
+      <c r="D57" s="18">
         <v>6.3</v>
       </c>
       <c r="E57" s="17">
@@ -3072,7 +3122,7 @@
       <c r="C58" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D58" s="19">
+      <c r="D58" s="18">
         <v>7.8</v>
       </c>
       <c r="E58" s="17">
@@ -3098,7 +3148,7 @@
       <c r="C59" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D59" s="19">
+      <c r="D59" s="18">
         <v>8.4</v>
       </c>
       <c r="E59" s="17">
@@ -3124,7 +3174,7 @@
       <c r="C60" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D60" s="19">
+      <c r="D60" s="18">
         <v>8.8000000000000007</v>
       </c>
       <c r="E60" s="17">
@@ -3150,7 +3200,7 @@
       <c r="C61" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="D61" s="19">
+      <c r="D61" s="18">
         <v>9.1999999999999993</v>
       </c>
       <c r="E61" s="17">
@@ -3188,14 +3238,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -3378,15 +3428,15 @@
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="18" t="s">
+      <c r="A15" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="18"/>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="19"/>
+      <c r="E15" s="19"/>
+      <c r="F15" s="19"/>
+      <c r="G15" s="19"/>
       <c r="H15" s="16"/>
     </row>
     <row r="16" spans="1:8" ht="14.4" thickBot="1" x14ac:dyDescent="0.3">

</xml_diff>